<commit_message>
Update Gantt_Proyecto_Graficacion.xlsx with new data
</commit_message>
<xml_diff>
--- a/Gantt_Proyecto_Graficacion.xlsx
+++ b/Gantt_Proyecto_Graficacion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nette\AppData\Local\Temp\claude\c--Users-nette-OneDrive-Documentos-Escuela-8vo-semestre-Graficaci-n-code\48bef41f-16ed-4090-9724-8ab7f9e359ee\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nette\OneDrive\Documentos\Escuela\8vo_semestre\Graficación\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74052D4F-ACCA-4033-A08E-6DF05653D10F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E28F99A-EBE0-450E-AA90-5E60CF9EC43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="1776" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt" sheetId="1" r:id="rId1"/>
@@ -186,18 +186,12 @@
     <t>Tarjetas de datos analíticos (pendiente, ecuación, incrementos)</t>
   </si>
   <si>
-    <t>Integración cálculo ↔ gráfica</t>
-  </si>
-  <si>
     <t>Sprint 3</t>
   </si>
   <si>
     <t>Tabla CTkTable con los puntos y pasos de la recta</t>
   </si>
   <si>
-    <t>Clasificación: 4 positivos, 4 negativos y 3 especiales (clasificar_recta)</t>
-  </si>
-  <si>
     <t>Recta vertical y punto único: cálculo y dibujo</t>
   </si>
   <si>
@@ -222,9 +216,6 @@
     <t>Modo Oscuro / Claro con CTkSwitch y sincronización del plano</t>
   </si>
   <si>
-    <t>Plano predominante (&gt;80 %) y ajuste responsivo</t>
-  </si>
-  <si>
     <t>Pruebas de navegación, interacción y regresión</t>
   </si>
   <si>
@@ -340,6 +331,15 @@
   </si>
   <si>
     <t>Total sprint</t>
+  </si>
+  <si>
+    <t>Plano predominante y ajuste responsivo</t>
+  </si>
+  <si>
+    <t>Clasificación: 4 positivos, 4 negativos y 3 especiales</t>
+  </si>
+  <si>
+    <t>Integración cálculo - gráfica</t>
   </si>
 </sst>
 </file>
@@ -654,7 +654,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill>
@@ -699,22 +699,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFE5E7EB"/>
           <bgColor rgb="FFE5E7EB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBD5D5"/>
-          <bgColor rgb="FFFBD5D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBD5D5"/>
-          <bgColor rgb="FFFBD5D5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3156,7 +3140,7 @@
         <v>34</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="C27" s="22" t="str">
         <f>Equipo!$B$5</f>
@@ -3211,7 +3195,7 @@
     </row>
     <row r="28" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B28" s="21" t="s">
         <v>28</v>
@@ -3269,10 +3253,10 @@
     </row>
     <row r="29" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="21" t="s">
         <v>41</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>42</v>
       </c>
       <c r="C29" s="22" t="str">
         <f>Equipo!$B$6</f>
@@ -3327,10 +3311,10 @@
     </row>
     <row r="30" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="C30" s="22" t="str">
         <f>Equipo!$B$6</f>
@@ -3385,10 +3369,10 @@
     </row>
     <row r="31" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C31" s="22" t="str">
         <f>Equipo!$B$5</f>
@@ -3443,10 +3427,10 @@
     </row>
     <row r="32" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C32" s="22" t="str">
         <f>Equipo!$B$5</f>
@@ -3501,10 +3485,10 @@
     </row>
     <row r="33" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C33" s="22" t="str">
         <f>Equipo!$B$7</f>
@@ -3559,10 +3543,10 @@
     </row>
     <row r="34" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C34" s="22" t="str">
         <f>Equipo!$B$7</f>
@@ -3617,7 +3601,7 @@
     </row>
     <row r="35" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B35" s="21" t="s">
         <v>28</v>
@@ -3675,10 +3659,10 @@
     </row>
     <row r="36" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C36" s="22" t="str">
         <f>Equipo!$B$6</f>
@@ -3733,10 +3717,10 @@
     </row>
     <row r="37" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="21" t="s">
         <v>48</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>50</v>
       </c>
       <c r="C37" s="22" t="str">
         <f>Equipo!$B$6</f>
@@ -3791,10 +3775,10 @@
     </row>
     <row r="38" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C38" s="22" t="str">
         <f>Equipo!$B$7</f>
@@ -3849,10 +3833,10 @@
     </row>
     <row r="39" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="C39" s="22" t="str">
         <f>Equipo!$B$5</f>
@@ -3907,10 +3891,10 @@
     </row>
     <row r="40" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C40" s="22" t="str">
         <f>Equipo!$B$5</f>
@@ -3965,10 +3949,10 @@
     </row>
     <row r="41" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C41" s="22" t="str">
         <f>Equipo!$B$7</f>
@@ -4023,10 +4007,10 @@
     </row>
     <row r="42" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C42" s="22" t="str">
         <f>Equipo!$B$8</f>
@@ -4081,10 +4065,10 @@
     </row>
     <row r="43" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C43" s="22" t="str">
         <f>Equipo!$B$8</f>
@@ -4148,7 +4132,7 @@
     <mergeCell ref="O6:U6"/>
   </mergeCells>
   <conditionalFormatting sqref="H7:AQ7">
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>WEEKDAY(H$8,2)&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4205,7 +4189,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4225,72 +4209,72 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="25" t="s">
         <v>59</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>63</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>67</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="28" t="s">
         <v>74</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -4307,7 +4291,7 @@
     </row>
     <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="32" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -4315,7 +4299,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B12" s="33">
         <v>46251</v>
@@ -4325,7 +4309,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B13" s="33">
         <v>46286</v>
@@ -4335,10 +4319,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -4368,7 +4352,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4394,22 +4378,22 @@
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="F4" s="17" t="s">
         <v>85</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -4492,7 +4476,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="40" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="41">
@@ -4530,7 +4514,7 @@
     </row>
     <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="32" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -4555,7 +4539,7 @@
         <v>Ulises Chauk Arias Santiz</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F12" s="2"/>
     </row>
@@ -4627,7 +4611,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="36">
         <f>SUMPRODUCT((Gantt!$A$9:$A$43=$A16)*(Gantt!$C$9:$C$43=B$12)*(Gantt!$E$9:$E$43-Gantt!$D$9:$D$43+1))-COUNTIFS(Gantt!$A$9:$A$43,$A16,Gantt!$C$9:$C$43,B$12,Gantt!$D$9:$D$43,"&lt;="&amp;DiaSinTrabajo,Gantt!$E$9:$E$43,"&gt;="&amp;DiaSinTrabajo)</f>
@@ -4649,7 +4633,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="40" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B17" s="36">
         <f>SUMPRODUCT((Gantt!$A$9:$A$43=$A17)*(Gantt!$C$9:$C$43=B$12)*(Gantt!$E$9:$E$43-Gantt!$D$9:$D$43+1))-COUNTIFS(Gantt!$A$9:$A$43,$A17,Gantt!$C$9:$C$43,B$12,Gantt!$D$9:$D$43,"&lt;="&amp;DiaSinTrabajo,Gantt!$E$9:$E$43,"&gt;="&amp;DiaSinTrabajo)</f>
@@ -4671,7 +4655,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="40" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B18" s="41">
         <f>SUM(B13:B17)</f>

</xml_diff>